<commit_message>
Re-verify issue tracker against the live site (2026-09-07): 0 of 239 fixed, 9 new findings added
Re-crawled all 86 content pages, re-checked all 143 internal link targets,
and re-probed the 32 junk/redirect/dead-link URLs individually. Every
tracked issue is still present exactly as described on 2026-09-03; nothing
has been fixed on the live site.

Two things changed since the original audit, neither a fix: a new page
went live (/brand-store-design/, thin content, no meta description, no
alt text) and a new junk taxonomy appeared (7 dsm-attachment-category
archive pages, indexable, same pattern as project_category). Added as
9 new tracker rows (AS-240 to AS-248), bringing the total to 248.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TbLUcNPxRUqBBBz7fDi7SJ
</commit_message>
<xml_diff>
--- a/seo-geo/tracking/issue-tracker.xlsx
+++ b/seo-geo/tracking/issue-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Issues" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues'!$A$1:$J$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues'!$A$1:$J$249</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,14 +439,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J240"/>
+  <dimension ref="A1:J249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
@@ -11978,10 +11978,442 @@
       </c>
       <c r="J240" s="2" t="inlineStr"/>
     </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>AS-240</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>New page: Brand Store Design</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/brand-store-design/</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>New page found live, not in the original audit: thin content, no meta description, no alt text</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/brand-store-design/ did not exist on 2026-09-03 (confirmed absent from the page sitemap that day) and is live as of the 2026-09-07 re-check: HTTP 200, in the page sitemap, published page count rose from 50 to 51. It has one H1 ("Brand Store Design"), 17 words of body copy, no meta description, and 48 of 48 images with empty alt text. It carries the same sitewide Organization/ProfessionalService schema as every other page (see the schema rows above), so it inherits that issue too.</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>Give this page the same treatment as the other primary pages: write a meta description, expand the body copy well past 17 words (what Brand Store design work includes, examples, a link to the portfolio gallery), and add alt text to all 48 images.</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>AS-241</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>New page: Brand Store Design</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/brand-store-design/</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>No call to action visible in the first mobile screen</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Rendered at 390x844, the only CTA ("Contact") is inside the collapsed nav menu, same pattern as most other pages.</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>Add a visible CTA button under the H1.</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>AS-242</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: ABG</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/abg/</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/abg/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>AS-243</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: BeYoutifull</t>
+        </is>
+      </c>
+      <c r="D244" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/beyoutifull/</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/beyoutifull/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>AS-244</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: Katjes</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/katjes/</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/katjes/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>AS-245</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: Magmod</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/magmod/</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/magmod/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>AS-246</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: Mouthwatchers</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/mouthwatchers/</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/mouthwatchers/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>AS-247</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: Rufus</t>
+        </is>
+      </c>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/rufus/</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/rufus/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>AS-248</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>New since 2026-09-03: dsm-attachment-category archives</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>DSM attachment category archive: Tabanero</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/tabanero/</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>New junk taxonomy archive found live and indexable, not present on 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>https://www.albertscott.com/blog/dsm-attachment-category/tabanero/ did not exist on 2026-09-03. As of 2026-09-07 it returns HTTP 200, self canonical, no noindex meta tag, and is listed in a new child sitemap at https://www.albertscott.com/dsm-attachment-category-sitemap.xml (7 URLs total, all named after client brands: ABG, BeYoutifull, Katjes, Magmod, Mouthwatchers, Rufus, Tabanero). This is the same pattern as the project_category archives already flagged: an auto-generated taxonomy archive with no unique content, here from a Divi Supreme Modules plugin feature.</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>In All in One SEO &gt; Search Appearance &gt; Taxonomies, find "DSM Attachment Category" (or the equivalent label the Divi Supreme Modules plugin registers) and set "Show in search results" to No and untick "Include in sitemap", the same fix already applied to the other taxonomy archives.</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J240"/>
+  <autoFilter ref="A1:J249"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J240" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Done,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12225,6 +12657,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId237"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId238"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId248"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>